<commit_message>
Add equipment_block supportedStructureType term; fix PB1-stale sourceElementXpath
New term for a heavy reinforced-concrete block/plinth foundation sized to a single piece of
substation or industrial equipment (a power transformer or shunt reactor, typically) - distinct
from mat, which is building-raft-flavored. Also fixes all 11 pre-existing entries' and the
dictionary's own description's sourceElementXpath/reference, still pointing at
diggs:RIProgramBasis after diggs-schema's PB1 moved supportedStructureType to
diggs:RILTPDesign - a follow-up PB1 missed since its own verification never searched def for
this element by name.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Codelist Excel Files and Conversion Templates to XML/supportedStructureType.xlsx
+++ b/Codelist Excel Files and Conversion Templates to XML/supportedStructureType.xlsx
@@ -985,7 +985,7 @@
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Codes naming what a rigid inclusion program supports - the load source the design is prepared for. Used for the value of the supportedStructureType property of diggs:RIProgramBasis, which RI_Design_Parameter_Analysis.md Group A row 4 identifies as the master conditional a large part of the Design and Post-installation parameter groups key on: several other properties are meaningful only for an embankment or wall, others only for a slab or mat. The list is open.</t>
+          <t>Codes naming what a load transfer platform supports - the load source the design is prepared for. Used for the value of the supportedStructureType property of diggs:RILTPDesign (moved off diggs:RIProgramBasis at PB1, 2026-09-23, once real project data - a nine-zone substation under one shared basis - showed the value varies per platform, not per program). Several other properties are meaningful only for an embankment or wall, others only for a slab or mat. The list is open.</t>
         </is>
       </c>
     </row>
@@ -1422,12 +1422,32 @@
         <f>IF(ISNA(VLOOKUP(B13,AssociatedElements!B$2:B2951,1,FALSE)),"Not used","")</f>
         <v/>
       </c>
-      <c r="B13" s="13" t="n"/>
-      <c r="C13" s="13" t="n"/>
-      <c r="D13" s="14" t="n"/>
-      <c r="E13" s="13" t="n"/>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>equipment_block</t>
+        </is>
+      </c>
+      <c r="C13" s="13" t="inlineStr">
+        <is>
+          <t>Heavy equipment block foundation</t>
+        </is>
+      </c>
+      <c r="D13" s="14" t="inlineStr">
+        <is>
+          <t>A heavy reinforced-concrete block or plinth foundation sized to a single piece of substation or industrial equipment - a power transformer or shunt reactor, typically - supported by the rigid inclusions and load transfer platform. Rigid and continuous like a mat, but distinct from it: sized to the equipment footprint rather than spanning a building's structural grid.</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
       <c r="F13" s="13" t="n"/>
-      <c r="G13" s="9" t="n"/>
+      <c r="G13" s="9" t="inlineStr">
+        <is>
+          <t>DIGGS</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2">
@@ -1764,7 +1784,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>//diggs:RIProgramBasis/diggs:supportedStructureType</t>
+          <t>//diggs:RILTPDesign/diggs:supportedStructureType</t>
         </is>
       </c>
     </row>
@@ -1780,7 +1800,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>//diggs:RIProgramBasis/diggs:supportedStructureType</t>
+          <t>//diggs:RILTPDesign/diggs:supportedStructureType</t>
         </is>
       </c>
     </row>
@@ -1796,7 +1816,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>//diggs:RIProgramBasis/diggs:supportedStructureType</t>
+          <t>//diggs:RILTPDesign/diggs:supportedStructureType</t>
         </is>
       </c>
     </row>
@@ -1812,7 +1832,7 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>//diggs:RIProgramBasis/diggs:supportedStructureType</t>
+          <t>//diggs:RILTPDesign/diggs:supportedStructureType</t>
         </is>
       </c>
     </row>
@@ -1828,7 +1848,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>//diggs:RIProgramBasis/diggs:supportedStructureType</t>
+          <t>//diggs:RILTPDesign/diggs:supportedStructureType</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1864,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>//diggs:RIProgramBasis/diggs:supportedStructureType</t>
+          <t>//diggs:RILTPDesign/diggs:supportedStructureType</t>
         </is>
       </c>
     </row>
@@ -1860,7 +1880,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>//diggs:RIProgramBasis/diggs:supportedStructureType</t>
+          <t>//diggs:RILTPDesign/diggs:supportedStructureType</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1896,7 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>//diggs:RIProgramBasis/diggs:supportedStructureType</t>
+          <t>//diggs:RILTPDesign/diggs:supportedStructureType</t>
         </is>
       </c>
     </row>
@@ -1892,7 +1912,7 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>//diggs:RIProgramBasis/diggs:supportedStructureType</t>
+          <t>//diggs:RILTPDesign/diggs:supportedStructureType</t>
         </is>
       </c>
     </row>
@@ -1908,7 +1928,7 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>//diggs:RIProgramBasis/diggs:supportedStructureType</t>
+          <t>//diggs:RILTPDesign/diggs:supportedStructureType</t>
         </is>
       </c>
     </row>
@@ -1924,7 +1944,7 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>//diggs:RIProgramBasis/diggs:supportedStructureType</t>
+          <t>//diggs:RILTPDesign/diggs:supportedStructureType</t>
         </is>
       </c>
     </row>
@@ -1933,7 +1953,16 @@
         <f>IF(ISNA(VLOOKUP(B13,Definitions!B$2:B$1839,1,FALSE)),"Not listed","")</f>
         <v/>
       </c>
-      <c r="B13" s="20" t="n"/>
+      <c r="B13" s="20" t="inlineStr">
+        <is>
+          <t>equipment_block</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>//diggs:RILTPDesign/diggs:supportedStructureType</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14">

</xml_diff>